<commit_message>
Vertaal alpha-statussen van Paved road en Governance naar het Nederlands
Sync EA_Alpha_Assessment.xlsx mee: Governance-labels vertaald, en de
Paved Road-sheet teruggebracht van 5 naar de 3 statussen die de RDF
kent (Seeded en Pervasive bestonden niet meer).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/essence/EA_Alpha_Assessment.xlsx
+++ b/essence/EA_Alpha_Assessment.xlsx
@@ -2130,7 +2130,7 @@
       </c>
       <c r="G12" s="107" t="inlineStr">
         <is>
-          <t>Pervasive</t>
+          <t>Evoluerend</t>
         </is>
       </c>
       <c r="H12" s="108">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="G20" s="107" t="inlineStr">
         <is>
-          <t>Effective</t>
+          <t>Effectief</t>
         </is>
       </c>
       <c r="H20" s="108">
@@ -2751,7 +2751,7 @@
     <row r="7" ht="35" customHeight="1" s="86">
       <c r="B7" s="157" t="inlineStr">
         <is>
-          <t>1. Initiated</t>
+          <t>1. Opgericht</t>
         </is>
       </c>
       <c r="C7" s="240" t="inlineStr">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="G7" s="85" t="inlineStr">
         <is>
-          <t>Initiated</t>
+          <t>Opgericht</t>
         </is>
       </c>
       <c r="H7" s="85">
@@ -2804,7 +2804,7 @@
       <c r="E8" s="161" t="n"/>
       <c r="G8" s="85" t="inlineStr">
         <is>
-          <t>Engaged</t>
+          <t>Actief</t>
         </is>
       </c>
       <c r="H8" s="85">
@@ -2826,7 +2826,7 @@
     <row r="9" ht="35" customHeight="1" s="86">
       <c r="B9" s="195" t="inlineStr">
         <is>
-          <t>2. Engaged</t>
+          <t>2. Actief</t>
         </is>
       </c>
       <c r="C9" s="235" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="G9" s="85" t="inlineStr">
         <is>
-          <t>Guiding</t>
+          <t>Sturend</t>
         </is>
       </c>
       <c r="H9" s="85">
@@ -2879,7 +2879,7 @@
       <c r="E10" s="161" t="n"/>
       <c r="G10" s="85" t="inlineStr">
         <is>
-          <t>Assured</t>
+          <t>Geborgd</t>
         </is>
       </c>
       <c r="H10" s="85">
@@ -2901,7 +2901,7 @@
     <row r="11" ht="35" customHeight="1" s="86">
       <c r="B11" s="157" t="inlineStr">
         <is>
-          <t>3. Guiding</t>
+          <t>3. Sturend</t>
         </is>
       </c>
       <c r="C11" s="240" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="G11" s="85" t="inlineStr">
         <is>
-          <t>Effective</t>
+          <t>Effectief</t>
         </is>
       </c>
       <c r="H11" s="85">
@@ -2956,7 +2956,7 @@
     <row r="13" ht="35" customHeight="1" s="86">
       <c r="B13" s="195" t="inlineStr">
         <is>
-          <t>4. Assured</t>
+          <t>4. Geborgd</t>
         </is>
       </c>
       <c r="C13" s="235" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="15" ht="35" customHeight="1" s="86">
       <c r="B15" s="157" t="inlineStr">
         <is>
-          <t>5. Effective</t>
+          <t>5. Effectief</t>
         </is>
       </c>
       <c r="C15" s="240" t="n"/>
@@ -4349,7 +4349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:M16"/>
+  <dimension ref="B1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="85" min="1" max="1"/>
@@ -4367,7 +4367,7 @@
         </is>
       </c>
       <c r="M1" s="85">
-        <f>SUM(H7:H11)</f>
+        <f>SUM(H7:H9)</f>
         <v/>
       </c>
     </row>
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="M2" s="85">
-        <f>SUM(I7:I11)</f>
+        <f>SUM(I7:I9)</f>
         <v/>
       </c>
     </row>
@@ -4394,7 +4394,7 @@
         </is>
       </c>
       <c r="M3" s="85">
-        <f>SUM(K7:K11)</f>
+        <f>SUM(K7:K9)</f>
         <v/>
       </c>
     </row>
@@ -4420,13 +4420,13 @@
         </is>
       </c>
       <c r="M4" s="85">
-        <f>SUM(J7:J11)</f>
+        <f>SUM(J7:J9)</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="25.5" customHeight="1" s="86">
       <c r="B5" s="182">
-        <f>IF(M3=0,"Not started",INDEX(G7:G11,M3))</f>
+        <f>IF(M3=0,"Not started",INDEX(G7:G9,M3))</f>
         <v/>
       </c>
       <c r="C5" s="183">
@@ -4434,7 +4434,7 @@
         <v/>
       </c>
       <c r="D5" s="182">
-        <f>M4&amp;" / "&amp;5</f>
+        <f>M4&amp;" / "&amp;3</f>
         <v/>
       </c>
       <c r="E5" s="184" t="inlineStr">
@@ -4468,7 +4468,7 @@
     <row r="7" ht="35" customHeight="1" s="86">
       <c r="B7" s="127" t="inlineStr">
         <is>
-          <t>1. Seeded</t>
+          <t>1. Vastgesteld</t>
         </is>
       </c>
       <c r="C7" s="233" t="inlineStr">
@@ -4478,7 +4478,7 @@
       </c>
       <c r="D7" s="220" t="inlineStr">
         <is>
-          <t>De behoefte aan een paved road wordt onderkend.</t>
+          <t>Een coherent service-chassis van goedgekeurde producten, patronen en standaarden is gepubliceerd.</t>
         </is>
       </c>
       <c r="E7" s="130">
@@ -4487,7 +4487,7 @@
       </c>
       <c r="G7" s="85" t="inlineStr">
         <is>
-          <t>Seeded</t>
+          <t>Vastgesteld</t>
         </is>
       </c>
       <c r="H7" s="85">
@@ -4515,13 +4515,13 @@
       </c>
       <c r="D8" s="208" t="inlineStr">
         <is>
-          <t>Een eerste goedgekeurde standaardkeuze of twee bestaat al.</t>
+          <t>De goedgekeurde route is zelfbedienbaar.</t>
         </is>
       </c>
       <c r="E8" s="131" t="n"/>
       <c r="G8" s="85" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Toegepast</t>
         </is>
       </c>
       <c r="H8" s="85">
@@ -4543,7 +4543,7 @@
     <row r="9" ht="35" customHeight="1" s="86">
       <c r="B9" s="185" t="inlineStr">
         <is>
-          <t>2. Established</t>
+          <t>2. Toegepast</t>
         </is>
       </c>
       <c r="C9" s="235" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="D9" s="223" t="inlineStr">
         <is>
-          <t>Een samenhangend service-chassis van goedgekeurde producten, patronen en standaarden is gepubliceerd.</t>
+          <t>Teams bouwen standaard op de goedgekeurde route.</t>
         </is>
       </c>
       <c r="E9" s="188">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="G9" s="85" t="inlineStr">
         <is>
-          <t>Adopted</t>
+          <t>Evoluerend</t>
         </is>
       </c>
       <c r="H9" s="85">
@@ -4583,158 +4583,62 @@
     </row>
     <row r="10" ht="35" customHeight="1" s="86">
       <c r="B10" s="131" t="n"/>
-      <c r="C10" s="236" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
+      <c r="C10" s="236" t="n"/>
       <c r="D10" s="210" t="inlineStr">
         <is>
-          <t>De paved road is zelfbedienbaar.</t>
+          <t>On-road keuzes hoeven niet te worden beoordeeld.</t>
         </is>
       </c>
       <c r="E10" s="131" t="n"/>
-      <c r="G10" s="85" t="inlineStr">
-        <is>
-          <t>Pervasive</t>
-        </is>
-      </c>
-      <c r="H10" s="85">
-        <f>COUNTIF(C13:C14,"✔")</f>
-        <v/>
-      </c>
-      <c r="I10" s="85" t="n">
-        <v>2</v>
-      </c>
-      <c r="J10" s="85">
-        <f>IF(H10=I10,1,0)</f>
-        <v/>
-      </c>
-      <c r="K10" s="85">
-        <f>J10*K9</f>
-        <v/>
-      </c>
+      <c r="G10" s="85" t="n"/>
+      <c r="H10" s="85" t="n"/>
+      <c r="I10" s="85" t="n"/>
+      <c r="J10" s="85" t="n"/>
+      <c r="K10" s="85" t="n"/>
     </row>
     <row r="11" ht="35" customHeight="1" s="86">
       <c r="B11" s="127" t="inlineStr">
         <is>
-          <t>3. Adopted</t>
-        </is>
-      </c>
-      <c r="C11" s="233" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
+          <t>3. Evoluerend</t>
+        </is>
+      </c>
+      <c r="C11" s="233" t="n"/>
       <c r="D11" s="220" t="inlineStr">
         <is>
-          <t>Teams bouwen standaard op de paved road.</t>
+          <t>De goedgekeurde route wordt continu verbreed en gesnoeid.</t>
         </is>
       </c>
       <c r="E11" s="130">
         <f>COUNTIF(C11:C12,"✔")&amp;" / 2"</f>
         <v/>
       </c>
-      <c r="G11" s="85" t="inlineStr">
-        <is>
-          <t>Evolving</t>
-        </is>
-      </c>
-      <c r="H11" s="85">
-        <f>COUNTIF(C15:C16,"✔")</f>
-        <v/>
-      </c>
-      <c r="I11" s="85" t="n">
-        <v>2</v>
-      </c>
-      <c r="J11" s="85">
-        <f>IF(H11=I11,1,0)</f>
-        <v/>
-      </c>
-      <c r="K11" s="85">
-        <f>J11*K10</f>
-        <v/>
-      </c>
+      <c r="G11" s="85" t="n"/>
+      <c r="H11" s="85" t="n"/>
+      <c r="I11" s="85" t="n"/>
+      <c r="J11" s="85" t="n"/>
+      <c r="K11" s="85" t="n"/>
     </row>
     <row r="12" ht="35" customHeight="1" s="86">
       <c r="B12" s="131" t="n"/>
       <c r="C12" s="234" t="n"/>
       <c r="D12" s="208" t="inlineStr">
         <is>
-          <t>On-road keuzes hoeven niet te worden beoordeeld.</t>
+          <t>Lessen uit beoordelingen worden er in teruggevoerd.</t>
         </is>
       </c>
       <c r="E12" s="131" t="n"/>
-    </row>
-    <row r="13" ht="35" customHeight="1" s="86">
-      <c r="B13" s="185" t="inlineStr">
-        <is>
-          <t>4. Pervasive</t>
-        </is>
-      </c>
-      <c r="C13" s="235" t="n"/>
-      <c r="D13" s="223" t="inlineStr">
-        <is>
-          <t>De paved road is de norm binnen het hele landschap.</t>
-        </is>
-      </c>
-      <c r="E13" s="188">
-        <f>COUNTIF(C13:C14,"✔")&amp;" / 2"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="35" customHeight="1" s="86">
-      <c r="B14" s="131" t="n"/>
-      <c r="C14" s="236" t="n"/>
-      <c r="D14" s="210" t="inlineStr">
-        <is>
-          <t>Afwijken van de paved road is de zeldzame, verantwoorde uitzondering.</t>
-        </is>
-      </c>
-      <c r="E14" s="131" t="n"/>
-    </row>
-    <row r="15" ht="35" customHeight="1" s="86">
-      <c r="B15" s="127" t="inlineStr">
-        <is>
-          <t>5. Evolving</t>
-        </is>
-      </c>
-      <c r="C15" s="233" t="n"/>
-      <c r="D15" s="220" t="inlineStr">
-        <is>
-          <t>De paved road wordt continu verbreed en gesnoeid.</t>
-        </is>
-      </c>
-      <c r="E15" s="130">
-        <f>COUNTIF(C15:C16,"✔")&amp;" / 2"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="35" customHeight="1" s="86">
-      <c r="B16" s="131" t="n"/>
-      <c r="C16" s="234" t="n"/>
-      <c r="D16" s="208" t="inlineStr">
-        <is>
-          <t>Lessen uit beoordelingen worden erin teruggevoerd.</t>
-        </is>
-      </c>
-      <c r="E16" s="131" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="12">
+  <mergeCells count="8">
     <mergeCell ref="B9:B10"/>
     <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="E13:E14"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="B11:B12"/>
     <mergeCell ref="E7:E8"/>
-    <mergeCell ref="E15:E16"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="E11:E12"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B15:B16"/>
   </mergeCells>
   <conditionalFormatting sqref="E7:E8">
     <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="3" text="" percent="0" bottom="0">

</xml_diff>